<commit_message>
Update interface for PiecewiseConstantParameter
</commit_message>
<xml_diff>
--- a/tests/workbooks/test_parameter.xlsx
+++ b/tests/workbooks/test_parameter.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebastian\01_GitHub\sschlenkrich\QuantLibXlOil\tests\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38B82B2B-220A-4EBB-BDD5-10A3328C443B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA00667C-B6F3-4F70-BF72-9A48C4E1E2B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14340" yWindow="-19695" windowWidth="21330" windowHeight="15900" xr2:uid="{45A6C063-5495-498A-86BB-E2019A1EF4EC}"/>
+    <workbookView xWindow="13530" yWindow="-19245" windowWidth="23175" windowHeight="16410" xr2:uid="{45A6C063-5495-498A-86BB-E2019A1EF4EC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -487,9 +487,17 @@
       <c r="B3">
         <v>1</v>
       </c>
+      <c r="C3">
+        <f>$B$2</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <f>$B$2</f>
         <v>2</v>
       </c>
     </row>
@@ -497,6 +505,10 @@
       <c r="B5">
         <v>3</v>
       </c>
+      <c r="C5">
+        <f>$B$2</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -506,6 +518,10 @@
         <f t="array" ref="B6">_xll.qlPositiveConstraint()</f>
         <v>⚡[test_parameter.xlsx]Sheet1!R6C2PositiveConstraint,A</v>
       </c>
+      <c r="C6">
+        <f>$B$2</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -530,7 +546,7 @@
         <v>4</v>
       </c>
       <c r="B11" t="str" cm="1">
-        <f t="array" ref="B11">_xll.qlPiecewiseConstantParameter(B3:B5,B6)</f>
+        <f t="array" ref="B11">_xll.qlPiecewiseConstantParameter(B3:B5,C3:C6,B6)</f>
         <v>⚡[test_parameter.xlsx]Sheet1!R11C2PiecewiseConstantParameter,A</v>
       </c>
     </row>
@@ -540,7 +556,7 @@
       </c>
       <c r="B13" cm="1">
         <f t="array" ref="B13">_xll.qlParameterParams(B9)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
@@ -549,7 +565,7 @@
       </c>
       <c r="B14" cm="1">
         <f t="array" ref="B14">_xll.qlParameterParams(B10)</f>
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
@@ -558,16 +574,16 @@
       </c>
       <c r="B15" cm="1">
         <f t="array" ref="B15:E15">TRANSPOSE(_xll.qlParameterParams(B11))</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C15">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D15">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E15">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
@@ -640,13 +656,13 @@
         <v>5</v>
       </c>
       <c r="C26">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D26">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E26">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>